<commit_message>
Respostas da dona: hero, CTA, faixa, beneficios
</commit_message>
<xml_diff>
--- a/REVISAO-CONTEUDO.xlsx
+++ b/REVISAO-CONTEUDO.xlsx
@@ -1,18 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27932"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3C3B14C-037F-4222-88B5-0901CA2909C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Textos por dobra" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Imagens" state="visible" r:id="rId5"/>
+    <sheet name="Textos por dobra" sheetId="1" r:id="rId1"/>
+    <sheet name="Imagens" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="171027"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="840" uniqueCount="198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1101" uniqueCount="230">
   <si>
     <t>#</t>
   </si>
@@ -606,26 +615,132 @@
   </si>
   <si>
     <t>dp8.jpg</t>
+  </si>
+  <si>
+    <t>Tirar esse div, está repetitivo com o 11/12</t>
+  </si>
+  <si>
+    <t>mais(+)10 mil</t>
+  </si>
+  <si>
+    <t>COMEÇAR AGORA  →  [https://pay.kiwify.com.br/U4n0qN7]</t>
+  </si>
+  <si>
+    <t>remover, repetitivo</t>
+  </si>
+  <si>
+    <t>alunas transformadas + 10 países - pensar em fazer outra faixa para os países</t>
+  </si>
+  <si>
+    <t>Depois de 13 anos como fisioterapeuta e instrutora de pilates criei um método que nenhuma aula convencional entrega. O pilates em casa reúne: alivio de dores, definição e força em um progrmama com progressão, segurança e acompanhamento real, feito para encaixar na sua rotina.</t>
+  </si>
+  <si>
+    <t>Alunas que já transformaram seus corpos com o metodo Pilates em Casa</t>
+  </si>
+  <si>
+    <t>Imagens de alunas a serem enviadas antes/depois filtro de imagem em codigo.</t>
+  </si>
+  <si>
+    <t>Voce vai entender que nunca teve resultado porque nunca treinou com um método de verdade</t>
+  </si>
+  <si>
+    <t>refazer a copy dessa parte, definir e desinchar com constancia não me agradam</t>
+  </si>
+  <si>
+    <t>1 ano para treinar no seu ritmo. Acesso quando quiser do Celular, tv, computador ou tablet. - revisar copy</t>
+  </si>
+  <si>
+    <t>Grupo de alunas onde você pode tirar duvidas, interagir com outras alunas e compartilhar seus resultados.  - revisar copy</t>
+  </si>
+  <si>
+    <t>prova social sugerida</t>
+  </si>
+  <si>
+    <t>Esclarecimento</t>
+  </si>
+  <si>
+    <t>Falta falar ou no hero mais sobre o pilates em casa em si, das aulas, como funciona o curso principal</t>
+  </si>
+  <si>
+    <t>Pilates para mulher com rotina real: aliviar as dores, secar e definir, em casa, com aulas curtas, progressivas e guiadas por fisioterapeuta.</t>
+  </si>
+  <si>
+    <t>copiar do site: https://elah-app.com/ - o script que faz 2 fotos antes e depois serem umas em cimas das outras, com filtro visual de antes/depois, logo abaixo do texto: Você entenderá que nunca teve resultado satisfatório porque nunca treinou com sistema de verdade.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">app da kiwify, imagem de referencia em </t>
+  </si>
+  <si>
+    <t>Um programa completo para você treinar em casa, no seu ritmo, com aulas guiadas e acesso a tudo pelo celular.</t>
+  </si>
+  <si>
+    <t>E faria os blocos assim:</t>
+  </si>
+  <si>
+    <t>✓ 28 aulas de Pilates gravadas</t>
+  </si>
+  <si>
+    <t>Aulas práticas e guiadas para você treinar quando quiser, de onde estiver.</t>
+  </si>
+  <si>
+    <t>✓ Evolua sem precisar trocar de programa</t>
+  </si>
+  <si>
+    <t>Você tem 1 ano de acesso para começar no seu ritmo e, depois, continuar com as aulas e intensificar seus treinos conforme evolui.</t>
+  </si>
+  <si>
+    <t>✓ Para diferentes níveis e idades</t>
+  </si>
+  <si>
+    <t>Aulas fáceis de acompanhar e adaptáveis para diferentes corpos, níveis de condicionamento e momentos da vida.</t>
+  </si>
+  <si>
+    <t>✓ Plataforma exclusiva</t>
+  </si>
+  <si>
+    <t>Todo o seu programa organizado em uma área de membros, para você encontrar suas aulas e materiais com facilidade.</t>
+  </si>
+  <si>
+    <t>✓ Aplicativo para treinar onde quiser</t>
+  </si>
+  <si>
+    <t>Acesse suas aulas pelo celular de forma prática, em casa, viajando ou onde estiver.</t>
+  </si>
+  <si>
+    <t>✓ Nunca treine sozinha</t>
+  </si>
+  <si>
+    <t>Conte com a orientação da Naty durante as aulas e tenha um espaço para tirar suas dúvidas e seguir sua evolução.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <i/>
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <b/>
-      <color rgb="FFFFFFFF"/>
-    </font>
-    <font>
-      <i/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -658,7 +773,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -672,6 +787,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1010,9 +1129,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F139"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:F160"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
@@ -1141,7 +1260,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1154,14 +1273,14 @@
       <c r="D7" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E7" s="3" t="s">
-        <v>9</v>
+      <c r="E7" s="7" t="s">
+        <v>213</v>
       </c>
       <c r="F7" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1174,8 +1293,8 @@
       <c r="D8" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="E8" s="3" t="s">
-        <v>9</v>
+      <c r="E8" s="8" t="s">
+        <v>203</v>
       </c>
       <c r="F8" t="s">
         <v>9</v>
@@ -1194,8 +1313,8 @@
       <c r="D9" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="E9" s="3" t="s">
-        <v>9</v>
+      <c r="E9" s="2" t="s">
+        <v>200</v>
       </c>
       <c r="F9" t="s">
         <v>9</v>
@@ -1215,7 +1334,7 @@
         <v>20</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>9</v>
+        <v>201</v>
       </c>
       <c r="F10" t="s">
         <v>9</v>
@@ -1235,7 +1354,7 @@
         <v>22</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>9</v>
+        <v>198</v>
       </c>
       <c r="F11" t="s">
         <v>9</v>
@@ -1255,7 +1374,7 @@
         <v>24</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>9</v>
+        <v>199</v>
       </c>
       <c r="F12" t="s">
         <v>9</v>
@@ -1275,7 +1394,7 @@
         <v>25</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>9</v>
+        <v>202</v>
       </c>
       <c r="F13" t="s">
         <v>9</v>
@@ -1354,9 +1473,7 @@
       <c r="D17" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="E17" s="3" t="s">
-        <v>9</v>
-      </c>
+      <c r="E17" s="3"/>
       <c r="F17" t="s">
         <v>9</v>
       </c>
@@ -1401,98 +1518,48 @@
         <v>9</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20">
-        <v>19</v>
-      </c>
-      <c r="B20" t="s">
-        <v>32</v>
-      </c>
-      <c r="C20" t="s">
-        <v>33</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>34</v>
-      </c>
+    <row r="20" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="D20" s="2"/>
       <c r="E20" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F20" t="s">
-        <v>9</v>
+        <v>214</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21">
-        <v>20</v>
-      </c>
-      <c r="B21" t="s">
-        <v>32</v>
-      </c>
-      <c r="C21" t="s">
-        <v>17</v>
-      </c>
       <c r="D21" s="2" t="s">
-        <v>35</v>
+        <v>210</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F21" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22">
-        <v>21</v>
-      </c>
-      <c r="B22" t="s">
-        <v>32</v>
-      </c>
-      <c r="C22" t="s">
-        <v>17</v>
-      </c>
+        <v>204</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="D22" s="2" t="s">
-        <v>36</v>
+        <v>210</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F22" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23">
-        <v>22</v>
-      </c>
-      <c r="B23" t="s">
-        <v>32</v>
-      </c>
-      <c r="C23" t="s">
-        <v>17</v>
-      </c>
+        <v>206</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="D23" s="2" t="s">
-        <v>37</v>
+        <v>210</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F23" t="s">
-        <v>9</v>
+        <v>205</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="B24" t="s">
         <v>32</v>
       </c>
       <c r="C24" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="E24" s="3" t="s">
         <v>9</v>
@@ -1503,39 +1570,37 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B25" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="C25" t="s">
         <v>17</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="E25" s="3" t="s">
-        <v>9</v>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="E25" s="2"/>
       <c r="F25" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B26" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="C26" t="s">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>9</v>
+        <v>215</v>
       </c>
       <c r="F26" t="s">
         <v>9</v>
@@ -1543,16 +1608,16 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B27" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="C27" t="s">
         <v>17</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="E27" s="3" t="s">
         <v>9</v>
@@ -1561,18 +1626,18 @@
         <v>9</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A28">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B28" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="C28" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="E28" s="3" t="s">
         <v>9</v>
@@ -1583,7 +1648,7 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B29" t="s">
         <v>39</v>
@@ -1592,7 +1657,7 @@
         <v>17</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="E29" s="3" t="s">
         <v>9</v>
@@ -1603,16 +1668,16 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B30" t="s">
         <v>39</v>
       </c>
       <c r="C30" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="E30" s="3" t="s">
         <v>9</v>
@@ -1621,9 +1686,9 @@
         <v>9</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A31">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B31" t="s">
         <v>39</v>
@@ -1632,7 +1697,7 @@
         <v>17</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="E31" s="3" t="s">
         <v>9</v>
@@ -1641,9 +1706,9 @@
         <v>9</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A32">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="B32" t="s">
         <v>39</v>
@@ -1652,18 +1717,18 @@
         <v>17</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>9</v>
+        <v>207</v>
       </c>
       <c r="F32" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A33">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="B33" t="s">
         <v>39</v>
@@ -1672,7 +1737,7 @@
         <v>17</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E33" s="3" t="s">
         <v>9</v>
@@ -1683,16 +1748,16 @@
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B34" t="s">
         <v>39</v>
       </c>
       <c r="C34" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>19</v>
+        <v>45</v>
       </c>
       <c r="E34" s="3" t="s">
         <v>9</v>
@@ -1701,38 +1766,38 @@
         <v>9</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A35">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B35" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="C35" t="s">
         <v>17</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="E35" s="3" t="s">
-        <v>9</v>
+        <v>46</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>208</v>
       </c>
       <c r="F35" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A36">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="B36" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="C36" t="s">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E36" s="3" t="s">
         <v>9</v>
@@ -1741,21 +1806,21 @@
         <v>9</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A37">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="B37" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="C37" t="s">
         <v>17</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="E37" s="3" t="s">
-        <v>9</v>
+        <v>48</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>209</v>
       </c>
       <c r="F37" t="s">
         <v>9</v>
@@ -1763,16 +1828,16 @@
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="B38" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="C38" t="s">
-        <v>53</v>
+        <v>7</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>54</v>
+        <v>19</v>
       </c>
       <c r="E38" s="3" t="s">
         <v>9</v>
@@ -1783,16 +1848,16 @@
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B39" t="s">
         <v>49</v>
       </c>
       <c r="C39" t="s">
-        <v>53</v>
+        <v>17</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="E39" s="3" t="s">
         <v>9</v>
@@ -1803,16 +1868,16 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="B40" t="s">
         <v>49</v>
       </c>
       <c r="C40" t="s">
-        <v>7</v>
+        <v>33</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>19</v>
+        <v>51</v>
       </c>
       <c r="E40" s="3" t="s">
         <v>9</v>
@@ -1821,18 +1886,18 @@
         <v>9</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A41">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="B41" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="C41" t="s">
         <v>17</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="E41" s="3" t="s">
         <v>9</v>
@@ -1843,16 +1908,16 @@
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B42" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="C42" t="s">
-        <v>33</v>
+        <v>53</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="E42" s="3" t="s">
         <v>9</v>
@@ -1863,16 +1928,16 @@
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B43" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="C43" t="s">
-        <v>17</v>
+        <v>53</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="E43" s="3" t="s">
         <v>9</v>
@@ -1883,16 +1948,16 @@
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="B44" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="C44" t="s">
-        <v>53</v>
+        <v>7</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>60</v>
+        <v>19</v>
       </c>
       <c r="E44" s="3" t="s">
         <v>9</v>
@@ -1903,7 +1968,7 @@
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B45" t="s">
         <v>56</v>
@@ -1912,7 +1977,7 @@
         <v>17</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="E45" s="3" t="s">
         <v>9</v>
@@ -1923,16 +1988,16 @@
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="B46" t="s">
         <v>56</v>
       </c>
       <c r="C46" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="E46" s="3" t="s">
         <v>9</v>
@@ -1943,16 +2008,16 @@
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B47" t="s">
         <v>56</v>
       </c>
       <c r="C47" t="s">
-        <v>53</v>
+        <v>17</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="E47" s="3" t="s">
         <v>9</v>
@@ -1963,16 +2028,16 @@
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="B48" t="s">
         <v>56</v>
       </c>
       <c r="C48" t="s">
-        <v>17</v>
+        <v>53</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="E48" s="3" t="s">
         <v>9</v>
@@ -1981,9 +2046,9 @@
         <v>9</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A49">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="B49" t="s">
         <v>56</v>
@@ -1992,7 +2057,7 @@
         <v>17</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="E49" s="3" t="s">
         <v>9</v>
@@ -2003,16 +2068,16 @@
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B50" t="s">
         <v>56</v>
       </c>
       <c r="C50" t="s">
-        <v>53</v>
+        <v>17</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="E50" s="3" t="s">
         <v>9</v>
@@ -2023,16 +2088,16 @@
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="B51" t="s">
         <v>56</v>
       </c>
       <c r="C51" t="s">
-        <v>17</v>
+        <v>53</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="E51" s="3" t="s">
         <v>9</v>
@@ -2043,7 +2108,7 @@
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B52" t="s">
         <v>56</v>
@@ -2052,7 +2117,7 @@
         <v>17</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="E52" s="3" t="s">
         <v>9</v>
@@ -2063,16 +2128,16 @@
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="B53" t="s">
         <v>56</v>
       </c>
       <c r="C53" t="s">
-        <v>53</v>
+        <v>17</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="E53" s="3" t="s">
         <v>9</v>
@@ -2083,16 +2148,16 @@
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="B54" t="s">
         <v>56</v>
       </c>
       <c r="C54" t="s">
-        <v>17</v>
+        <v>53</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="E54" s="3" t="s">
         <v>9</v>
@@ -2101,9 +2166,9 @@
         <v>9</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A55">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="B55" t="s">
         <v>56</v>
@@ -2112,7 +2177,7 @@
         <v>17</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E55" s="3" t="s">
         <v>9</v>
@@ -2123,16 +2188,16 @@
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="B56" t="s">
         <v>56</v>
       </c>
       <c r="C56" t="s">
-        <v>53</v>
+        <v>17</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="E56" s="3" t="s">
         <v>9</v>
@@ -2143,16 +2208,16 @@
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="B57" t="s">
         <v>56</v>
       </c>
       <c r="C57" t="s">
-        <v>17</v>
+        <v>53</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="E57" s="3" t="s">
         <v>9</v>
@@ -2163,7 +2228,7 @@
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B58" t="s">
         <v>56</v>
@@ -2172,7 +2237,7 @@
         <v>17</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="E58" s="3" t="s">
         <v>9</v>
@@ -2183,16 +2248,16 @@
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="B59" t="s">
         <v>56</v>
       </c>
       <c r="C59" t="s">
-        <v>53</v>
+        <v>17</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="E59" s="3" t="s">
         <v>9</v>
@@ -2203,16 +2268,16 @@
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="B60" t="s">
         <v>56</v>
       </c>
       <c r="C60" t="s">
-        <v>17</v>
+        <v>53</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="E60" s="3" t="s">
         <v>9</v>
@@ -2223,7 +2288,7 @@
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="B61" t="s">
         <v>56</v>
@@ -2232,7 +2297,7 @@
         <v>17</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E61" s="3" t="s">
         <v>9</v>
@@ -2243,16 +2308,16 @@
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="B62" t="s">
         <v>56</v>
       </c>
       <c r="C62" t="s">
-        <v>53</v>
+        <v>17</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>76</v>
+        <v>62</v>
       </c>
       <c r="E62" s="3" t="s">
         <v>9</v>
@@ -2263,16 +2328,16 @@
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="B63" t="s">
         <v>56</v>
       </c>
       <c r="C63" t="s">
-        <v>17</v>
+        <v>53</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="E63" s="3" t="s">
         <v>9</v>
@@ -2283,7 +2348,7 @@
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B64" t="s">
         <v>56</v>
@@ -2292,7 +2357,7 @@
         <v>17</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E64" s="3" t="s">
         <v>9</v>
@@ -2303,16 +2368,16 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="B65" t="s">
         <v>56</v>
       </c>
       <c r="C65" t="s">
-        <v>53</v>
+        <v>17</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E65" s="3" t="s">
         <v>9</v>
@@ -2323,16 +2388,16 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="B66" t="s">
         <v>56</v>
       </c>
       <c r="C66" t="s">
-        <v>17</v>
+        <v>53</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="E66" s="3" t="s">
         <v>9</v>
@@ -2343,7 +2408,7 @@
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="B67" t="s">
         <v>56</v>
@@ -2352,7 +2417,7 @@
         <v>17</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="E67" s="3" t="s">
         <v>9</v>
@@ -2363,16 +2428,16 @@
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="B68" t="s">
         <v>56</v>
       </c>
       <c r="C68" t="s">
-        <v>53</v>
+        <v>17</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="E68" s="3" t="s">
         <v>9</v>
@@ -2383,16 +2448,16 @@
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="B69" t="s">
         <v>56</v>
       </c>
       <c r="C69" t="s">
-        <v>17</v>
+        <v>53</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="E69" s="3" t="s">
         <v>9</v>
@@ -2401,9 +2466,9 @@
         <v>9</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A70">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="B70" t="s">
         <v>56</v>
@@ -2412,7 +2477,7 @@
         <v>17</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="E70" s="3" t="s">
         <v>9</v>
@@ -2423,16 +2488,16 @@
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B71" t="s">
         <v>56</v>
       </c>
       <c r="C71" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>19</v>
+        <v>80</v>
       </c>
       <c r="E71" s="3" t="s">
         <v>9</v>
@@ -2443,16 +2508,16 @@
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B72" t="s">
-        <v>83</v>
+        <v>56</v>
       </c>
       <c r="C72" t="s">
-        <v>33</v>
+        <v>53</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="E72" s="3" t="s">
         <v>9</v>
@@ -2461,18 +2526,18 @@
         <v>9</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A73">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="B73" t="s">
-        <v>83</v>
+        <v>56</v>
       </c>
       <c r="C73" t="s">
         <v>17</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="E73" s="3" t="s">
         <v>9</v>
@@ -2483,16 +2548,16 @@
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="B74" t="s">
-        <v>83</v>
+        <v>56</v>
       </c>
       <c r="C74" t="s">
-        <v>86</v>
+        <v>17</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="E74" s="3" t="s">
         <v>9</v>
@@ -2503,16 +2568,16 @@
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B75" t="s">
-        <v>83</v>
+        <v>56</v>
       </c>
       <c r="C75" t="s">
-        <v>86</v>
+        <v>7</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>88</v>
+        <v>19</v>
       </c>
       <c r="E75" s="3" t="s">
         <v>9</v>
@@ -2523,16 +2588,16 @@
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="B76" t="s">
         <v>83</v>
       </c>
       <c r="C76" t="s">
-        <v>86</v>
+        <v>33</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="E76" s="3" t="s">
         <v>9</v>
@@ -2541,18 +2606,18 @@
         <v>9</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A77">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="B77" t="s">
         <v>83</v>
       </c>
       <c r="C77" t="s">
-        <v>86</v>
+        <v>17</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="E77" s="3" t="s">
         <v>9</v>
@@ -2563,7 +2628,7 @@
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="B78" t="s">
         <v>83</v>
@@ -2572,7 +2637,7 @@
         <v>86</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="E78" s="3" t="s">
         <v>9</v>
@@ -2583,7 +2648,7 @@
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B79" t="s">
         <v>83</v>
@@ -2592,7 +2657,7 @@
         <v>86</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="E79" s="3" t="s">
         <v>9</v>
@@ -2603,7 +2668,7 @@
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B80" t="s">
         <v>83</v>
@@ -2612,7 +2677,7 @@
         <v>86</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="E80" s="3" t="s">
         <v>9</v>
@@ -2623,7 +2688,7 @@
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="B81" t="s">
         <v>83</v>
@@ -2632,7 +2697,7 @@
         <v>86</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="E81" s="3" t="s">
         <v>9</v>
@@ -2643,7 +2708,7 @@
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="B82" t="s">
         <v>83</v>
@@ -2652,7 +2717,7 @@
         <v>86</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="E82" s="3" t="s">
         <v>9</v>
@@ -2663,7 +2728,7 @@
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="B83" t="s">
         <v>83</v>
@@ -2672,7 +2737,7 @@
         <v>86</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="E83" s="3" t="s">
         <v>9</v>
@@ -2683,16 +2748,16 @@
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="B84" t="s">
         <v>83</v>
       </c>
       <c r="C84" t="s">
-        <v>17</v>
+        <v>86</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="E84" s="3" t="s">
         <v>9</v>
@@ -2703,16 +2768,16 @@
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="B85" t="s">
         <v>83</v>
       </c>
       <c r="C85" t="s">
-        <v>17</v>
+        <v>86</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="E85" s="3" t="s">
         <v>9</v>
@@ -2723,16 +2788,16 @@
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="B86" t="s">
         <v>83</v>
       </c>
       <c r="C86" t="s">
-        <v>17</v>
+        <v>86</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="E86" s="3" t="s">
         <v>9</v>
@@ -2743,16 +2808,16 @@
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B87" t="s">
         <v>83</v>
       </c>
       <c r="C87" t="s">
-        <v>7</v>
+        <v>86</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>19</v>
+        <v>96</v>
       </c>
       <c r="E87" s="3" t="s">
         <v>9</v>
@@ -2763,7 +2828,7 @@
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="B88" t="s">
         <v>83</v>
@@ -2772,7 +2837,7 @@
         <v>17</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="E88" s="3" t="s">
         <v>9</v>
@@ -2783,16 +2848,16 @@
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="B89" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="C89" t="s">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="E89" s="3" t="s">
         <v>9</v>
@@ -2803,16 +2868,16 @@
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B90" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="C90" t="s">
-        <v>103</v>
+        <v>17</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="E90" s="3" t="s">
         <v>9</v>
@@ -2823,16 +2888,16 @@
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B91" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="C91" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>105</v>
+        <v>19</v>
       </c>
       <c r="E91" s="3" t="s">
         <v>9</v>
@@ -2841,18 +2906,18 @@
         <v>9</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A92">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B92" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="C92" t="s">
-        <v>106</v>
+        <v>17</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="E92" s="3" t="s">
         <v>9</v>
@@ -2863,16 +2928,16 @@
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B93" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="C93" t="s">
         <v>33</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="E93" s="3" t="s">
         <v>9</v>
@@ -2881,18 +2946,18 @@
         <v>9</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A94">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B94" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="C94" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="E94" s="3" t="s">
         <v>9</v>
@@ -2901,18 +2966,18 @@
         <v>9</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A95">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="B95" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="C95" t="s">
         <v>17</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="E95" s="3" t="s">
         <v>9</v>
@@ -2923,16 +2988,16 @@
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="B96" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="C96" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="E96" s="3" t="s">
         <v>9</v>
@@ -2943,16 +3008,16 @@
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B97" t="s">
         <v>108</v>
       </c>
       <c r="C97" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="E97" s="3" t="s">
         <v>9</v>
@@ -2963,7 +3028,7 @@
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="B98" t="s">
         <v>108</v>
@@ -2972,7 +3037,7 @@
         <v>110</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="E98" s="3" t="s">
         <v>9</v>
@@ -2981,9 +3046,9 @@
         <v>9</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A99">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="B99" t="s">
         <v>108</v>
@@ -2992,7 +3057,7 @@
         <v>17</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="E99" s="3" t="s">
         <v>9</v>
@@ -3003,7 +3068,7 @@
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="B100" t="s">
         <v>108</v>
@@ -3012,7 +3077,7 @@
         <v>110</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="E100" s="3" t="s">
         <v>9</v>
@@ -3021,9 +3086,9 @@
         <v>9</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A101">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="B101" t="s">
         <v>108</v>
@@ -3032,7 +3097,7 @@
         <v>17</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="E101" s="3" t="s">
         <v>9</v>
@@ -3043,7 +3108,7 @@
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A102">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="B102" t="s">
         <v>108</v>
@@ -3052,7 +3117,7 @@
         <v>110</v>
       </c>
       <c r="D102" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="E102" s="3" t="s">
         <v>9</v>
@@ -3061,9 +3126,9 @@
         <v>9</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A103">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="B103" t="s">
         <v>108</v>
@@ -3072,7 +3137,7 @@
         <v>17</v>
       </c>
       <c r="D103" s="2" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="E103" s="3" t="s">
         <v>9</v>
@@ -3083,7 +3148,7 @@
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A104">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="B104" t="s">
         <v>108</v>
@@ -3092,7 +3157,7 @@
         <v>110</v>
       </c>
       <c r="D104" s="2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="E104" s="3" t="s">
         <v>9</v>
@@ -3101,9 +3166,9 @@
         <v>9</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A105">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="B105" t="s">
         <v>108</v>
@@ -3112,7 +3177,7 @@
         <v>17</v>
       </c>
       <c r="D105" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="E105" s="3" t="s">
         <v>9</v>
@@ -3123,7 +3188,7 @@
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A106">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="B106" t="s">
         <v>108</v>
@@ -3132,7 +3197,7 @@
         <v>110</v>
       </c>
       <c r="D106" s="2" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="E106" s="3" t="s">
         <v>9</v>
@@ -3141,9 +3206,9 @@
         <v>9</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A107">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="B107" t="s">
         <v>108</v>
@@ -3152,7 +3217,7 @@
         <v>17</v>
       </c>
       <c r="D107" s="2" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="E107" s="3" t="s">
         <v>9</v>
@@ -3163,7 +3228,7 @@
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A108">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="B108" t="s">
         <v>108</v>
@@ -3172,7 +3237,7 @@
         <v>110</v>
       </c>
       <c r="D108" s="2" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="E108" s="3" t="s">
         <v>9</v>
@@ -3181,9 +3246,9 @@
         <v>9</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A109">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="B109" t="s">
         <v>108</v>
@@ -3192,7 +3257,7 @@
         <v>17</v>
       </c>
       <c r="D109" s="2" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="E109" s="3" t="s">
         <v>9</v>
@@ -3203,7 +3268,7 @@
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A110">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="B110" t="s">
         <v>108</v>
@@ -3212,7 +3277,7 @@
         <v>110</v>
       </c>
       <c r="D110" s="2" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="E110" s="3" t="s">
         <v>9</v>
@@ -3221,9 +3286,9 @@
         <v>9</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A111">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B111" t="s">
         <v>108</v>
@@ -3232,7 +3297,7 @@
         <v>17</v>
       </c>
       <c r="D111" s="2" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="E111" s="3" t="s">
         <v>9</v>
@@ -3243,7 +3308,7 @@
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A112">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="B112" t="s">
         <v>108</v>
@@ -3252,7 +3317,7 @@
         <v>110</v>
       </c>
       <c r="D112" s="2" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="E112" s="3" t="s">
         <v>9</v>
@@ -3261,9 +3326,9 @@
         <v>9</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A113">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="B113" t="s">
         <v>108</v>
@@ -3272,7 +3337,7 @@
         <v>17</v>
       </c>
       <c r="D113" s="2" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="E113" s="3" t="s">
         <v>9</v>
@@ -3283,7 +3348,7 @@
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A114">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="B114" t="s">
         <v>108</v>
@@ -3292,7 +3357,7 @@
         <v>110</v>
       </c>
       <c r="D114" s="2" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="E114" s="3" t="s">
         <v>9</v>
@@ -3303,7 +3368,7 @@
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A115">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="B115" t="s">
         <v>108</v>
@@ -3312,7 +3377,7 @@
         <v>17</v>
       </c>
       <c r="D115" s="2" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="E115" s="3" t="s">
         <v>9</v>
@@ -3323,16 +3388,16 @@
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A116">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="B116" t="s">
-        <v>133</v>
+        <v>108</v>
       </c>
       <c r="C116" t="s">
-        <v>33</v>
+        <v>110</v>
       </c>
       <c r="D116" s="2" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="E116" s="3" t="s">
         <v>9</v>
@@ -3341,18 +3406,18 @@
         <v>9</v>
       </c>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A117">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="B117" t="s">
-        <v>133</v>
+        <v>108</v>
       </c>
       <c r="C117" t="s">
         <v>17</v>
       </c>
       <c r="D117" s="2" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="E117" s="3" t="s">
         <v>9</v>
@@ -3363,16 +3428,16 @@
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A118">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="B118" t="s">
-        <v>133</v>
+        <v>108</v>
       </c>
       <c r="C118" t="s">
-        <v>7</v>
+        <v>110</v>
       </c>
       <c r="D118" s="2" t="s">
-        <v>19</v>
+        <v>131</v>
       </c>
       <c r="E118" s="3" t="s">
         <v>9</v>
@@ -3381,18 +3446,18 @@
         <v>9</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A119">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="B119" t="s">
-        <v>133</v>
+        <v>108</v>
       </c>
       <c r="C119" t="s">
         <v>17</v>
       </c>
       <c r="D119" s="2" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="E119" s="3" t="s">
         <v>9</v>
@@ -3403,16 +3468,16 @@
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A120">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="B120" t="s">
         <v>133</v>
       </c>
       <c r="C120" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="D120" s="2" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="E120" s="3" t="s">
         <v>9</v>
@@ -3421,18 +3486,18 @@
         <v>9</v>
       </c>
     </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A121">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="B121" t="s">
         <v>133</v>
       </c>
       <c r="C121" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="D121" s="2" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="E121" s="3" t="s">
         <v>9</v>
@@ -3443,7 +3508,7 @@
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A122">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="B122" t="s">
         <v>133</v>
@@ -3452,7 +3517,7 @@
         <v>7</v>
       </c>
       <c r="D122" s="2" t="s">
-        <v>139</v>
+        <v>19</v>
       </c>
       <c r="E122" s="3" t="s">
         <v>9</v>
@@ -3461,18 +3526,18 @@
         <v>9</v>
       </c>
     </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A123">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="B123" t="s">
         <v>133</v>
       </c>
       <c r="C123" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="D123" s="2" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="E123" s="3" t="s">
         <v>9</v>
@@ -3483,16 +3548,16 @@
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A124">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="B124" t="s">
         <v>133</v>
       </c>
       <c r="C124" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="D124" s="2" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="E124" s="3" t="s">
         <v>9</v>
@@ -3503,7 +3568,7 @@
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A125">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="B125" t="s">
         <v>133</v>
@@ -3512,7 +3577,7 @@
         <v>7</v>
       </c>
       <c r="D125" s="2" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="E125" s="3" t="s">
         <v>9</v>
@@ -3521,18 +3586,18 @@
         <v>9</v>
       </c>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A126">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B126" t="s">
         <v>133</v>
       </c>
       <c r="C126" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="D126" s="2" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="E126" s="3" t="s">
         <v>9</v>
@@ -3543,16 +3608,16 @@
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A127">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="B127" t="s">
         <v>133</v>
       </c>
       <c r="C127" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="D127" s="2" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="E127" s="3" t="s">
         <v>9</v>
@@ -3563,7 +3628,7 @@
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A128">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="B128" t="s">
         <v>133</v>
@@ -3572,7 +3637,7 @@
         <v>7</v>
       </c>
       <c r="D128" s="2" t="s">
-        <v>19</v>
+        <v>141</v>
       </c>
       <c r="E128" s="3" t="s">
         <v>9</v>
@@ -3583,16 +3648,16 @@
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A129">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="B129" t="s">
-        <v>145</v>
+        <v>133</v>
       </c>
       <c r="C129" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="D129" s="2" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="E129" s="3" t="s">
         <v>9</v>
@@ -3603,16 +3668,16 @@
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A130">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="B130" t="s">
-        <v>145</v>
+        <v>133</v>
       </c>
       <c r="C130" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="D130" s="2" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="E130" s="3" t="s">
         <v>9</v>
@@ -3623,16 +3688,16 @@
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A131">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="B131" t="s">
-        <v>145</v>
+        <v>133</v>
       </c>
       <c r="C131" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="D131" s="2" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="E131" s="3" t="s">
         <v>9</v>
@@ -3643,16 +3708,16 @@
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A132">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B132" t="s">
-        <v>145</v>
+        <v>133</v>
       </c>
       <c r="C132" t="s">
         <v>7</v>
       </c>
       <c r="D132" s="2" t="s">
-        <v>140</v>
+        <v>19</v>
       </c>
       <c r="E132" s="3" t="s">
         <v>9</v>
@@ -3663,16 +3728,16 @@
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A133">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="B133" t="s">
         <v>145</v>
       </c>
       <c r="C133" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="D133" s="2" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="E133" s="3" t="s">
         <v>9</v>
@@ -3683,7 +3748,7 @@
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A134">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="B134" t="s">
         <v>145</v>
@@ -3692,7 +3757,7 @@
         <v>7</v>
       </c>
       <c r="D134" s="2" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="E134" s="3" t="s">
         <v>9</v>
@@ -3701,18 +3766,18 @@
         <v>9</v>
       </c>
     </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A135">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="B135" t="s">
         <v>145</v>
       </c>
       <c r="C135" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="D135" s="2" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="E135" s="3" t="s">
         <v>9</v>
@@ -3723,16 +3788,16 @@
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A136">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="B136" t="s">
         <v>145</v>
       </c>
       <c r="C136" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="D136" s="2" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="E136" s="3" t="s">
         <v>9</v>
@@ -3743,7 +3808,7 @@
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A137">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="B137" t="s">
         <v>145</v>
@@ -3752,33 +3817,194 @@
         <v>7</v>
       </c>
       <c r="D137" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="E137" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F137" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="138" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A138">
+        <v>133</v>
+      </c>
+      <c r="B138" t="s">
+        <v>145</v>
+      </c>
+      <c r="C138" t="s">
+        <v>7</v>
+      </c>
+      <c r="D138" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="E138" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F138" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="139" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A139">
+        <v>134</v>
+      </c>
+      <c r="B139" t="s">
+        <v>145</v>
+      </c>
+      <c r="C139" t="s">
+        <v>17</v>
+      </c>
+      <c r="D139" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="E139" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F139" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="140" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A140">
+        <v>135</v>
+      </c>
+      <c r="B140" t="s">
+        <v>145</v>
+      </c>
+      <c r="C140" t="s">
+        <v>17</v>
+      </c>
+      <c r="D140" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="E140" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F140" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="141" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A141">
+        <v>136</v>
+      </c>
+      <c r="B141" t="s">
+        <v>145</v>
+      </c>
+      <c r="C141" t="s">
+        <v>7</v>
+      </c>
+      <c r="D141" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="E137" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F137" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="139" spans="2:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B139" s="4" t="s">
+      <c r="E141" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F141" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="143" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B143" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="D139" s="4" t="s">
+      <c r="D143" s="4" t="s">
         <v>147</v>
+      </c>
+    </row>
+    <row r="145" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B145" t="s">
+        <v>211</v>
+      </c>
+      <c r="D145" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="147" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B147" t="s">
+        <v>211</v>
+      </c>
+      <c r="D147" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="148" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="D148" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="149" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="D149" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="150" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="D150" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="151" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="D151" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="152" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="D152" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="153" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="D153" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="154" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="D154" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="155" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="D155" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="156" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="D156" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="157" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="D157" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="158" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="D158" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="159" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="D159" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="160" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="D160" t="s">
+        <v>229</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:D38"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
@@ -4320,6 +4546,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>